<commit_message>
Ajout de production et financement
</commit_message>
<xml_diff>
--- a/Documentation dashboards.xlsx
+++ b/Documentation dashboards.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unionhabitat.sharepoint.com/sites/Directiondesetudes/Documents partages/General/Direction/Projets/SI DATA/01 - Projet datawarehouse/10 - Documentation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ykraiem\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="270" documentId="8_{E38240D2-6D03-460C-AD1F-56A7CB9B1EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92565F34-EE0C-4D23-9F15-D94300D44B3F}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{411B2BE2-86D3-43AC-A02C-4AB7B88665B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53012F43-4FC2-4F6E-9064-525D4764D57E}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="3795" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{78D94C61-402A-46A6-8F9B-6154C169E404}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Description" sheetId="3" r:id="rId1"/>
-    <sheet name="Indicateurs" sheetId="1" r:id="rId2"/>
-    <sheet name="Axes d'analyses" sheetId="2" r:id="rId3"/>
+    <sheet name="Description" sheetId="1" r:id="rId1"/>
+    <sheet name="Indicateurs" sheetId="2" r:id="rId2"/>
+    <sheet name="Axes d'analyses" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="258">
   <si>
     <t>Theme</t>
   </si>
@@ -95,6 +95,26 @@
     <t>SNE, INSEE</t>
   </si>
   <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>L'objectif est de présenter, pour chaque territoire, le volume de logements sociaux agréés dans l'année, leur répartition par type de financement (PLAI dont PLAI adapté, PLUS, PLS), par mode de production (construction neuve, acquisition-amélioration, acquisition sans travaux) et par nature du logement (ordinaire ou spécifique). Les typologies de logements (T1 à T5 et plus) sont également présentées.
+Les engagements dans le cadre du Programme National de Renouvellement Urbain (ANRU) font l'objet d'un traitement distinct et sont présentés séparément des opérations de droit commun. Seules les opérations de France métropolitaine et des régions d'Outre-Mer sont couvertes.</t>
+  </si>
+  <si>
+    <t>SIAP</t>
+  </si>
+  <si>
+    <t>Toutes les régions de France y compris les régions d'Outre-Mer</t>
+  </si>
+  <si>
+    <t>Financement</t>
+  </si>
+  <si>
+    <t>L'objectif est de présenter, pour chaque territoire, les coûts des opérations agréées dans l'année (coût global TTC et HT, coût par logement, coût au m²) ainsi que la décomposition du financement selon sa source : fonds propres de l'organisme, emprunts (prêts Caisse des Dépôts et assimilés) et subventions (État, collectivités territoriales, Action Logement et autres aides publiques). La part du foncier dans le coût global est également documentée.
+Les opérations ANRU sont exclues du périmètre. Seules les opérations de France métropolitaine et des régions d'Outre-Mer sont couvertes.</t>
+  </si>
+  <si>
     <t>Indicateur</t>
   </si>
   <si>
@@ -207,6 +227,9 @@
 Les régions d'outre-mer sont exclus du calcul puisque le DPE GES n'est pas renseigné</t>
   </si>
   <si>
+    <t>Part de locataires sociaux</t>
+  </si>
+  <si>
     <t>Calcul: Nombre de logements sociaux occupés / Nombre de résidences principales privées</t>
   </si>
   <si>
@@ -269,6 +292,9 @@
     <t>Moyenne de l'ancienneté de la demande au 31 décembre de l'année selectionnée. Il s'agit donc de l'écart entre le jour de la demande de logement social et le 31 décembre de l'année sélectionnée</t>
   </si>
   <si>
+    <t>,</t>
+  </si>
+  <si>
     <t>Pression de la demande</t>
   </si>
   <si>
@@ -333,6 +359,227 @@
   </si>
   <si>
     <t>Rapport entre le nombre de logements attribués sur l'année sélectionnée et le nombre de demande en stock à fin de l'année sélectionnée</t>
+  </si>
+  <si>
+    <t>Nombre d'agréments hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre total de logements sociaux ayant obtenu un agrément de financement au cours de l'année de référence, hors opérations du Programme National de Renouvellement Urbain (ANRU).
+Calcul : somme des agréments par opération.</t>
+  </si>
+  <si>
+    <t>Nombre de logements ordinaires hors ANRU</t>
+  </si>
+  <si>
+    <t>Parmi les logements agréés, nombre de logements à usage de résidence principale ordinaire, à l'exclusion des logements spécifiques (foyers de jeunes travailleurs, résidences sociales, pensions de famille, logements adaptés). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de logements spécifiques hors ANRU</t>
+  </si>
+  <si>
+    <t>Parmi les logements agréés, nombre de logements à destination spécifique : résidences sociales, foyers de jeunes travailleurs, pensions de famille, logements adaptés aux personnes en situation de handicap ou âgées. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de PLAI hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés sous financement PLAI (Prêt Locatif Aidé d'Intégration), dont PLAI adapté. Le PLAI s'adresse aux ménages aux ressources très modestes et impose les niveaux de loyer les plus bas du parc social. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de PLAI adapté hors ANRU</t>
+  </si>
+  <si>
+    <t>Sous-ensemble du PLAI destiné aux personnes en très grande difficulté d'insertion sociale, dont le profil nécessite un accompagnement social renforcé. Ce volume est inclus dans le total PLAI. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de PLUS hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés sous financement PLUS (Prêt Locatif à Usage Social), financement de droit commun du logement social accessible à la majorité des ménages. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de PLS hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés sous financement PLS (Prêt Locatif Social). Le PLS s'adresse aux ménages dont les ressources dépassent les plafonds PLUS et dont les loyers sont intermédiaires entre le parc HLM classique et le marché privé. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de construction neuve hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés produits par construction sur terrain nu (ex nihilo). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre d'acquisition-amélioration hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés produits par l'acquisition d'un bâtiment existant accompagnée de travaux de réhabilitation significatifs. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre d'acquisition sans travaux hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés produits par l'acquisition d'un bâtiment existant sans réalisation de travaux. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de T1 hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés de type T1 (une pièce principale). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de T2 hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés de type T2 (deux pièces principales). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de T3 hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés de type T3 (trois pièces principales). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de T4 hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés de type T4 (quatre pièces principales). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de T5 et plus hors ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés de type T5 et plus (cinq pièces principales et plus). Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre d'engagements ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements sociaux agréés dans le cadre d'opérations du Programme National de Renouvellement Urbain (ANRU). Présenté séparément des agréments de droit commun.</t>
+  </si>
+  <si>
+    <t>Nombre de PLAI ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements PLAI agréés dans le cadre d'opérations ANRU.</t>
+  </si>
+  <si>
+    <t>Nombre de PLUS ANRU</t>
+  </si>
+  <si>
+    <t>Nombre de logements PLUS agréés dans le cadre d'opérations ANRU.</t>
+  </si>
+  <si>
+    <t>Total (Agréments + engagements)</t>
+  </si>
+  <si>
+    <t>Volume total de logements sociaux produits dans l'année : somme des agréments hors ANRU et des engagements ANRU.
+Calcul : Nombre d'agréments hors ANRU + Nombre d'engagements ANRU.</t>
+  </si>
+  <si>
+    <t>Coût global de l'opération hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Montant total toutes taxes comprises de l'ensemble des opérations de production agréées dans l'année, hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût global de l'opération hors ANRU HT</t>
+  </si>
+  <si>
+    <t>Montant total hors taxes de l'ensemble des opérations de production agréées dans l'année, hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût de construction moyen hors ANRU TTC par logement</t>
+  </si>
+  <si>
+    <t>Coût moyen de l'opération TTC par logement agréé, calculé en rapportant le coût global TTC au nombre total d'agréments.
+Calcul : Coût global TTC / Nombre d'agréments hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût de construction médian hors ANRU TTC par logement</t>
+  </si>
+  <si>
+    <t>Médiane des coûts TTC par logement, calculée opération par opération. Moins sensible aux opérations atypiques que la moyenne, la médiane est l'indicateur de référence pour comparer les coûts de production entre territoires. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût de construction moyen hors ANRU TTC par m²</t>
+  </si>
+  <si>
+    <t>Coût moyen de construction TTC par m² de surface utile, calculé sur les opérations dont la surface est renseignée. Hors ANRU.
+Calcul : somme des coûts TTC des opérations à surface renseignée / surface utile totale de ces opérations.</t>
+  </si>
+  <si>
+    <t>Coût du foncier hors ANRU HT</t>
+  </si>
+  <si>
+    <t>Montant total hors taxes consacré à l'acquisition du foncier pour l'ensemble des opérations agréées dans l'année. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Part du foncier hors ANRU</t>
+  </si>
+  <si>
+    <t>Part du coût foncier dans le coût global HT des opérations agréées. Indicateur permettant d'apprécier la pression foncière par territoire.
+Calcul : Coût du foncier HT / Coût global HT.</t>
+  </si>
+  <si>
+    <t>Coût du bâtiment hors ANRU HT</t>
+  </si>
+  <si>
+    <t>Montant total hors taxes des travaux de construction ou de réhabilitation du bâtiment pour l'ensemble des opérations agréées dans l'année. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût des prestations intellectuelles hors ANRU HT</t>
+  </si>
+  <si>
+    <t>Montant total hors taxes des honoraires (maîtrise d'œuvre, études techniques, contrôle technique, assurances...) pour l'ensemble des opérations agréées. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Montant Fonds propres hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Montant total TTC financé par les fonds propres de l'organisme bailleur pour les opérations agréées dans l'année. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Montant Prêts hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Montant total TTC des emprunts contractés (prêts de la Caisse des Dépôts, prêts bancaires, prêts Action Logement...) pour les opérations agréées. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût de construction moyen emprunts hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Part des emprunts dans le financement, ramenée au logement. Calcul : Montant total des prêts TTC / Nombre d'agréments hors ANRU.</t>
+  </si>
+  <si>
+    <t>Montant Subventions hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Montant total TTC des subventions reçues — État (aides à la pierre), collectivités territoriales, Action Logement, autres financeurs publics — pour les opérations agréées dans l'année. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût source de financement hors ANRU TTC</t>
+  </si>
+  <si>
+    <t>Montant TTC apporté par la source de financement sélectionnée (fonds propres, prêts ou subventions) pour les opérations agréées, hors ANRU. Utilisé en combinaison avec le filtre par source de financement pour décomposer la structure de financement.</t>
+  </si>
+  <si>
+    <t>Nombre d'agréments hors ANRU (financement)</t>
+  </si>
+  <si>
+    <t>Nombre de logements agréés calculé depuis la table de financement, en agrégeant les données par opération et par source de financement. Donne le même résultat que le total Production mais depuis la table de financement. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Coût global de l'opération hors ANRU TTC (financement)</t>
+  </si>
+  <si>
+    <t>Montant total TTC ventilé par source de financement pour les opérations agréées dans l'année. Permet l'analyse du coût par source de financement. Hors ANRU.</t>
+  </si>
+  <si>
+    <t>Surface utile totale en m² hors ANRU</t>
+  </si>
+  <si>
+    <t>Somme des surfaces utiles en m² des logements agréés dans l'année. Hors ANRU.</t>
   </si>
   <si>
     <t>Axe</t>
@@ -603,22 +850,28 @@
 Radiation pour cause de non renouvellement</t>
   </si>
   <si>
-    <t>Part de locataires sociaux</t>
-  </si>
-  <si>
     <t>DALO</t>
   </si>
   <si>
+    <t>Demandeurs et attributaires reconnus prioritaires au titre DALO</t>
+  </si>
+  <si>
+    <t>Il s'agit d'une demande ou d'une attribution DALO ssi :
+- le statut dalo est différent de NON
+- le statut dalo n'est pas null
+- la date de décision dalo &lt;= 31/12/N</t>
+  </si>
+  <si>
     <t>Premier quartile</t>
   </si>
   <si>
+    <t>Demandeurs et attributaires dont les ressources se situent sous le premier quartile de ressources sur les territoires concernés par la réforme des attributions</t>
+  </si>
+  <si>
+    <t>Il s'agit d'une demande ou d'une attribution Premier quartile ssi (montant du revenu mensuel du foyer / unité de consommation) x 12 mois &lt;= montant du seuil de ressources</t>
+  </si>
+  <si>
     <t>Logement d'abord</t>
-  </si>
-  <si>
-    <t>Demandeurs et attributaires reconnus prioritaires au titre DALO</t>
-  </si>
-  <si>
-    <t>Demandeurs et attributaires dont les ressources se situent sous le premier quartile de ressources sur les territoires concernés par la réforme des attributions</t>
   </si>
   <si>
     <t>Demandeurs et attributaires bénéficiant du plan Logement d'abord</t>
@@ -636,20 +889,83 @@
 - Coordination thérapeutique</t>
   </si>
   <si>
-    <t>Il s'agit d'une demande ou d'une attribution Premier quartile ssi (montant du revenu mensuel du foyer / unité de consommation) x 12 mois &lt;= montant du seuil de ressources</t>
-  </si>
-  <si>
-    <t>Il s'agit d'une demande ou d'une attribution DALO ssi :
-- le statut dalo est différent de NON
-- le statut dalo n'est pas null
-- la date de décision dalo &lt;= 31/12/N</t>
+    <t>Mode de production</t>
+  </si>
+  <si>
+    <t>Mode de réalisation technique de l'opération de production de logements sociaux.</t>
+  </si>
+  <si>
+    <t>Construction neuve : logements construits sur terrain nu
+Acquisition-amélioration : acquisition d'un bâtiment existant avec travaux
+Acquisition sans travaux : achat d'un bâtiment existant sans réhabilitation
+Autre</t>
+  </si>
+  <si>
+    <t>Mode d'acquisition</t>
+  </si>
+  <si>
+    <t>Modalité juridique d'acquisition du foncier ou du bâti pour la réalisation de l'opération.</t>
+  </si>
+  <si>
+    <t>Construction sur terrain acquis · VEFA (Vente en État Futur d'Achèvement) · Bail emphytéotique · Bail à construction · Acquisition directe · Autre</t>
+  </si>
+  <si>
+    <t>Nature du logement</t>
+  </si>
+  <si>
+    <t>Catégorie du logement produit selon sa destination et sa réglementation.</t>
+  </si>
+  <si>
+    <t>Logement ordinaire : logement locatif social à usage de résidence principale
+Logement spécifique : résidence sociale, foyer de jeunes travailleurs, pension de famille, résidence étudiante
+Logement adapté : adapté aux personnes en situation de handicap ou âgées</t>
+  </si>
+  <si>
+    <t>Type de financement public accordé à l'opération. Détermine le niveau de loyer maximal et les plafonds de ressources des locataires.</t>
+  </si>
+  <si>
+    <t>PLAI : Prêt Locatif Aidé d'Intégration (ménages très modestes)
+PLUS : Prêt Locatif à Usage Social (financement de droit commun)
+PLS : Prêt Locatif Social (ménages aux revenus intermédiaires)
+Autres financements aidés</t>
+  </si>
+  <si>
+    <t>Type de bénéficiaire</t>
+  </si>
+  <si>
+    <t>Catégorie de l'organisme maître d'ouvrage bénéficiaire de l'agrément de production.</t>
+  </si>
+  <si>
+    <t>ESH (Entreprise Sociale pour l'Habitat / SA HLM) · OPH (Office Public de l'Habitat) · Coopérative HLM · SEM (Société d'Économie Mixte) · Organisme agréé · Autre</t>
+  </si>
+  <si>
+    <t>ANRU / Hors ANRU</t>
+  </si>
+  <si>
+    <t>Segmentation permettant de distinguer les opérations relevant du Programme National de Renouvellement Urbain (ANRU) de celles de droit commun.</t>
+  </si>
+  <si>
+    <t>ANRU : opérations engagées dans le cadre du renouvellement urbain
+Hors ANRU : opérations de droit commun
+Total : ANRU + Hors ANRU</t>
+  </si>
+  <si>
+    <t>Source de financement</t>
+  </si>
+  <si>
+    <t>Organisme ou dispositif ayant apporté un financement à l'opération de production. Trois grandes catégories sont distinguées selon la nature du financement.</t>
+  </si>
+  <si>
+    <t>Fonds propres : apport direct de l'organisme bailleur social
+Emprunts : prêts de la Caisse des Dépôts, prêts bancaires, prêts Action Logement
+Subventions : aides à la pierre de l'État, subventions des collectivités territoriales, aides Action Logement, autres aides publiques</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -725,9 +1041,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -743,6 +1059,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1077,15 +1394,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF32A818-55DC-4C7D-829B-81D7B53E1994}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10.3984375" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
     <col min="2" max="2" width="109" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1109,7 +1426,7 @@
       </c>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:8" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="128.25" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1130,7 +1447,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="85.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1151,431 +1468,872 @@
         <v>12</v>
       </c>
     </row>
+    <row r="4" spans="1:8" ht="85.5">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="71.25">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{EAB25B75-F1A1-4ADD-A90A-A502A052CA55}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{4C3DA737-6F2E-421C-84D3-2B4B25E9F2D7}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C998C4-4C13-4862-92D5-F4E9358593F6}">
-  <dimension ref="A1:C37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G73"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="18.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="73.59765625" customWidth="1"/>
-    <col min="4" max="4" width="10.73046875" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="65.5703125" customWidth="1"/>
+    <col min="3" max="3" width="73.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="42.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="42.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="42.75" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="57" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="71.25" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="57" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="71.25" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="28.5" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="57" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="57" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="42.75" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="85.5" x14ac:dyDescent="0.45">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="85.5" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="57" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="57" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="57" x14ac:dyDescent="0.45">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="57" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="42.75" customHeight="1">
+      <c r="A19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="28.5" customHeight="1">
+      <c r="A20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="71.25" customHeight="1">
+      <c r="A22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="57" customHeight="1">
+      <c r="A25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="42.75" customHeight="1">
+      <c r="A26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="28.5" customHeight="1">
+      <c r="A34" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="28.5" customHeight="1">
+      <c r="A37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="57">
+      <c r="A38" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="42.75">
+      <c r="A39" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="42.75">
+      <c r="A40" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="42.75">
+      <c r="A41" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="42.75">
+      <c r="A42" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="42.75">
+      <c r="A43" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="42.75">
+      <c r="A44" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="28.5">
+      <c r="A46" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="28.5">
+      <c r="A47" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="28.5">
+      <c r="A53" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="42.75">
+      <c r="A56" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="28.5">
+      <c r="A57" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="28.5">
+      <c r="A58" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="42.75">
+      <c r="A59" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="42.75">
+      <c r="A60" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="57">
+      <c r="A61" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="28.5">
+      <c r="A62" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="42.75">
+      <c r="A63" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="28.5">
+      <c r="A64" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A22" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="57" x14ac:dyDescent="0.45">
-      <c r="A25" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A28" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A31" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A34" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A35" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A36" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>88</v>
+      <c r="C64" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="28.5">
+      <c r="A65" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="28.5">
+      <c r="A66" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="28.5">
+      <c r="A67" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="28.5">
+      <c r="A68" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="42.75">
+      <c r="A69" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="42.75">
+      <c r="A70" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="42.75">
+      <c r="A71" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="28.5">
+      <c r="A72" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -1584,387 +2342,526 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D63C1C-82A7-4D8E-A65D-B74419366C15}">
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:E37"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="33.59765625" customWidth="1"/>
-    <col min="3" max="3" width="34.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.265625" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="33.5703125" customWidth="1"/>
+    <col min="3" max="3" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>89</v>
+        <v>169</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="85.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>91</v>
+        <v>171</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="28.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>94</v>
+        <v>174</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>95</v>
+        <v>175</v>
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="42.75" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>96</v>
+        <v>176</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>97</v>
+        <v>177</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="114" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="128.25" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>103</v>
+        <v>183</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="57" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>105</v>
+        <v>185</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>106</v>
+        <v>186</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="99.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>108</v>
+        <v>188</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>109</v>
+        <v>189</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="99.75" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>111</v>
+        <v>191</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>112</v>
+        <v>192</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="171" x14ac:dyDescent="0.45">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="171" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>114</v>
+        <v>194</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>115</v>
+        <v>195</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="187.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="187.5" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>118</v>
+        <v>198</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>119</v>
+        <v>199</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="85.5" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>201</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>122</v>
+        <v>202</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="270.75" x14ac:dyDescent="0.45">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="270.75" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>124</v>
+        <v>204</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>125</v>
+        <v>205</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="57" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>127</v>
+        <v>207</v>
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:5" ht="171" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="171" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>128</v>
+        <v>208</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>129</v>
+        <v>209</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="285" x14ac:dyDescent="0.45">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="285" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>131</v>
+        <v>211</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>132</v>
+        <v>212</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="85.5" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>134</v>
+        <v>214</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>135</v>
+        <v>215</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="242.25" x14ac:dyDescent="0.45">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="242.25" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>137</v>
+        <v>217</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>138</v>
+        <v>218</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="71.25" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>140</v>
+        <v>220</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>141</v>
+        <v>221</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="99.75" x14ac:dyDescent="0.45">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="99.75" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>143</v>
+        <v>223</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>144</v>
+        <v>224</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="85.5" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>146</v>
+        <v>226</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>147</v>
+        <v>227</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="71.25" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>150</v>
+        <v>229</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>153</v>
+        <v>230</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="57" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>151</v>
+        <v>232</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>154</v>
+        <v>233</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="171" x14ac:dyDescent="0.45">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="171" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>152</v>
+        <v>235</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C26" s="5"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C27" s="5"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C28" s="5"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C29" s="5"/>
-    </row>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="85.5">
+      <c r="A25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="42.75">
+      <c r="A26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="85.5">
+      <c r="A27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="57">
+      <c r="A28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="42.75">
+      <c r="A29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="57">
+      <c r="A30" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="85.5">
+      <c r="A31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="85.5">
+      <c r="A32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="42.75">
+      <c r="A33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="85.5">
+      <c r="A34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="57">
+      <c r="A35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="42.75">
+      <c r="A36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Sous_x002d_th_x00e8_me xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
-    <Ann_x00e9_e xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
-    <Donn_x00e9_esmobilis_x00e9_es xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
-    <Th_x00e8_me xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a63d3f7d-9ae7-4881-a2e5-01650a8247b9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052237A89E8CA214B92381756AEA23611" ma:contentTypeVersion="20" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="510f2d890aca16c7e52118f19c292bce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44042f46-c638-40f0-b803-0a3c16db3a5d" xmlns:ns3="a63d3f7d-9ae7-4881-a2e5-01650a8247b9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f5bb1233f2449b16a4f87373320f89a9" ns2:_="" ns3:_="">
     <xsd:import namespace="44042f46-c638-40f0-b803-0a3c16db3a5d"/>
@@ -2264,7 +3161,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2273,40 +3170,29 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Sous_x002d_th_x00e8_me xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
+    <Ann_x00e9_e xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
+    <Donn_x00e9_esmobilis_x00e9_es xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
+    <Th_x00e8_me xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44042f46-c638-40f0-b803-0a3c16db3a5d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a63d3f7d-9ae7-4881-a2e5-01650a8247b9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB5A1737-75AC-4C46-9CF2-0725CB708A15}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44042f46-c638-40f0-b803-0a3c16db3a5d"/>
-    <ds:schemaRef ds:uri="a63d3f7d-9ae7-4881-a2e5-01650a8247b9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8E4D90C-A9A5-4A73-BF8C-EEF74536E875}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C7AC71B-59C7-4E14-BBB6-8E6DAC860991}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="44042f46-c638-40f0-b803-0a3c16db3a5d"/>
-    <ds:schemaRef ds:uri="a63d3f7d-9ae7-4881-a2e5-01650a8247b9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1D2635B-B916-4E34-9AB4-DDDBD286E60B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F53CA91-B762-4110-8F3F-3FE1EDA322A6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7409EEEE-5CCC-44DE-BA4D-C67E7030C62B}"/>
 </file>
</xml_diff>